<commit_message>
Integrate Ashar PID: 17/17 PASS after 5 source-verified corrections; inventory 57 rows; regen workbook/DOCX/patch/package
</commit_message>
<xml_diff>
--- a/submission_pkg/24i3102_24i3052_24i3072_C_Workbook.xlsx
+++ b/submission_pkg/24i3102_24i3052_24i3072_C_Workbook.xlsx
@@ -44,13 +44,27 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
       <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00B0B0B0"/>
+      </left>
+      <right style="thin">
+        <color rgb="00B0B0B0"/>
+      </right>
+      <top style="thin">
+        <color rgb="00B0B0B0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00B0B0B0"/>
+      </bottom>
     </border>
   </borders>
   <cellStyleXfs count="1">
@@ -61,7 +75,7 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -429,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H52"/>
+  <dimension ref="A1:H58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -455,7 +469,7 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Purpose or scenario</t>
+          <t>Purpose / scenario</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
@@ -470,17 +484,17 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Execution result</t>
+          <t>Exec</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Structural-coverage target</t>
+          <t>Structural target</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Test-file / evidence reference</t>
+          <t>Ref</t>
         </is>
       </c>
     </row>
@@ -2172,22 +2186,22 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>updateIntegral</t>
+          <t>update + updateIntegral</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>non-finite integral candidate guarded</t>
+          <t>integral frozen when flag cleared, then evolves</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>fb +Inf, dt 0.1, I 0.1, sp 1</t>
+          <t>P2/I5, sp1, fb0, dt0.1, flag F then T</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>NaN output, integral stays 0; then normal ramp 0/0/0.01</t>
+          <t>2.0 + int 0; then 2.0 + int 0.5</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
@@ -2197,12 +2211,12 @@
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>P-D2 F-path</t>
+          <t>P-D1 F→T</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>NonFiniteIntegralGuarded</t>
+          <t>IntegralFrozenWhenUpdateFlagCleared</t>
         </is>
       </c>
     </row>
@@ -2214,22 +2228,22 @@
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>updateDerivative</t>
+          <t>output clamp + integral</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>guard all-false (dt 0, last NaN)</t>
+          <t>high-side saturation clamps output, integral accumulates (no freeze gate in v1.17.0)</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>fb 0.5, dt 0, D 5</t>
+          <t>I.5/lim10/out±.2, sp2, fb0, dt.5 ×2</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>0 + int.5; then .2 + int 1.0</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
@@ -2239,12 +2253,12 @@
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>P-D3 FF</t>
+          <t>saturation edges</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>DerivativeGuardAllFalse</t>
+          <t>SaturationHighClampsOutputIntegralNotFrozen</t>
         </is>
       </c>
     </row>
@@ -2256,22 +2270,22 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>updateDerivative</t>
+          <t>output clamp + integral</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>time ok, no history (dt 0.1, last NaN)</t>
+          <t>low-side mirror</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>fb 0.5, dt 0.1, D 5</t>
+          <t>sp−2 mirror</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>0 + int−.5; then −.2 + int −1.0</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
@@ -2281,12 +2295,12 @@
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>P-D3 TF</t>
+          <t>saturation edges</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>...TimeOkButNoHistory</t>
+          <t>SaturationLowClampsOutputIntegralNotFrozen</t>
         </is>
       </c>
     </row>
@@ -2298,22 +2312,22 @@
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>updateDerivative</t>
+          <t>integral unwind</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>fully active</t>
+          <t>error reversal under saturation unwinds integral</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>fb 0.5→0.6, dt 0.1, D 5</t>
+          <t>saturated-high, then sp→−2</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>5.0</t>
+          <t>.2 + int 0.5</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
@@ -2323,12 +2337,12 @@
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>P-D3 TT</t>
+          <t>saturation edges</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>...FullyActive</t>
+          <t>SaturationHighThenReversalUnwindsIntegral</t>
         </is>
       </c>
     </row>
@@ -2340,22 +2354,22 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>updateDerivative</t>
+          <t>updateIntegral</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>no time but history (dt 0, last finite)</t>
+          <t>NaN feedback discards integral candidate</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>fb 0.7, dt 0, D 5</t>
+          <t>P1/I.1, sp1, fb NaN</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>NaN out + int 0; then 0 + int 0</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
@@ -2365,12 +2379,12 @@
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>P-D3 FT</t>
+          <t>P-D2 F-path</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>...NoTimeButHistory</t>
+          <t>NonFiniteIntegralCandidateIsDiscarded_NaN</t>
         </is>
       </c>
     </row>
@@ -2382,22 +2396,22 @@
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>updateDerivative</t>
+          <t>updateIntegral + output clamp</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>exact dt==FLT_EPSILON boundary</t>
+          <t>−Inf feedback clamps output, integral held</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>dt FLT_EPSILON</t>
+          <t>P1/I.1, sp1, fb −Inf</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>0 (not &gt;)</t>
+          <t>+10 + int 0; then 0 + int 0</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
@@ -2407,12 +2421,12 @@
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>P-D3 boundary</t>
+          <t>P-D2 F-path + clamp</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
-          <t>...ExactEpsilonBoundary</t>
+          <t>..._NegInfSaturates</t>
         </is>
       </c>
     </row>
@@ -2429,17 +2443,17 @@
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>just above epsilon saturates via D</t>
+          <t>guard all-false (dt 0, last NaN)</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>dt 2*eps, D 5, limit 10</t>
+          <t>D4, fb2.0, dt0, fresh</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>10.0</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
@@ -2449,12 +2463,12 @@
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>P-D3 T + saturation</t>
+          <t>P-D3 FF</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
-          <t>...JustAboveEpsilonSaturates</t>
+          <t>DerivativeGuardBlocksWhenNoTimeAndNoHistory</t>
         </is>
       </c>
     </row>
@@ -2471,17 +2485,17 @@
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>negative dt robustness</t>
+          <t>time ok, no history (dt .5, last NaN)</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>dt -0.1, P 2</t>
+          <t>D4, fb2.0, dt.5, fresh</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>1.0 (P-only)</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
@@ -2491,12 +2505,12 @@
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>P-D3 invalid input</t>
+          <t>P-D3 TF</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr">
         <is>
-          <t>NegativeDtDisablesDerivative</t>
+          <t>...TimeOkButNoHistory</t>
         </is>
       </c>
     </row>
@@ -2508,22 +2522,22 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>resetDerivative</t>
+          <t>updateDerivative</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>history cleared to NaN</t>
+          <t>fully active (PLUS sign, L47)</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>reset then dt 0.1</t>
+          <t>D4, seed 2.0/.5, then 2.5/.5</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>+4.0</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
@@ -2533,12 +2547,12 @@
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>P-D3 TF re-entry</t>
+          <t>P-D3 TT</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
-          <t>ResetDerivativeClearsHistory</t>
+          <t>...ActiveWhenTimeAndHistory</t>
         </is>
       </c>
     </row>
@@ -2550,22 +2564,22 @@
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>updateIntegral</t>
+          <t>updateDerivative</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>windup clamps exactly at limit</t>
+          <t>history present but dt 0</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>I 1, lim 0.5, e 1, dt 0.5 ×3</t>
+          <t>D4, seed 2.0/.5, then 3.0/dt0</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>0, 0.5, 0.5; integral 0.5</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
@@ -2575,12 +2589,12 @@
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>P-D1 T + clamp</t>
+          <t>P-D3 FT</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr">
         <is>
-          <t>IntegralWindupClampsAtLimit</t>
+          <t>...HistoryButNoTime</t>
         </is>
       </c>
     </row>
@@ -2592,37 +2606,289 @@
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>update/output limit</t>
+          <t>updateDerivative</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
+          <t>exact dt==EPS boundary (not &gt;)</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>D4, seed 2.0/.5, then 2.5/dt=EPS</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G52" s="2" t="inlineStr">
+        <is>
+          <t>P-D3 boundary</t>
+        </is>
+      </c>
+      <c r="H52" s="2" t="inlineStr">
+        <is>
+          <t>...ExactEpsilonIsNotEnoughTime</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>PST-12</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>updateDerivative</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>just above EPS saturates high via D</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>D4, 2.5/dt=2EPS, lim±100</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="inlineStr">
+        <is>
+          <t>+100 (deriv 2097152 exact)</t>
+        </is>
+      </c>
+      <c r="F53" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G53" s="2" t="inlineStr">
+        <is>
+          <t>P-D3 T + saturation</t>
+        </is>
+      </c>
+      <c r="H53" s="2" t="inlineStr">
+        <is>
+          <t>...JustAboveEpsilonSaturatesHigh</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>PST-13</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>updateDerivative</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>negative dt robustness</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>P2/D4, sp1, fb.5, dt−.5</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>1.0 (P-only)</t>
+        </is>
+      </c>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G54" s="2" t="inlineStr">
+        <is>
+          <t>P-D3 invalid input</t>
+        </is>
+      </c>
+      <c r="H54" s="2" t="inlineStr">
+        <is>
+          <t>NegativeDtDisablesDerivativeTerm</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>PST-14</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>resetDerivative</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>history cleared to NaN, guard re-entry</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>D2, seed 0/.5, reset, then 1.0/.5</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F55" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G55" s="2" t="inlineStr">
+        <is>
+          <t>P-D3 TF re-entry</t>
+        </is>
+      </c>
+      <c r="H55" s="2" t="inlineStr">
+        <is>
+          <t>ResetDerivativeClearsHistory</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>PST-15</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>updateIntegral</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>windup clamps exactly at limit</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>I1/lim.5/out±10, sp1, fb0, dt.5 ×3</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t>0, .5, .5; int .5</t>
+        </is>
+      </c>
+      <c r="F56" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G56" s="2" t="inlineStr">
+        <is>
+          <t>P-D1 T + clamp</t>
+        </is>
+      </c>
+      <c r="H56" s="2" t="inlineStr">
+        <is>
+          <t>IntegralWindupClampsExactlyAtLimit</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>PST-16</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>output limit</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
           <t>exact-boundary passthrough + clamp</t>
         </is>
       </c>
-      <c r="D52" s="2" t="inlineStr">
-        <is>
-          <t>P 1, lim 2, sp 5, fb 3/2/4</t>
-        </is>
-      </c>
-      <c r="E52" s="2" t="inlineStr">
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>P1/lim±2, sp5, fb 3/2/4</t>
+        </is>
+      </c>
+      <c r="E57" s="2" t="inlineStr">
         <is>
           <t>2.0 / 2.0 / 1.0</t>
         </is>
       </c>
-      <c r="F52" s="2" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="G52" s="2" t="inlineStr">
+      <c r="F57" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G57" s="2" t="inlineStr">
         <is>
           <t>saturation edges</t>
         </is>
       </c>
-      <c r="H52" s="2" t="inlineStr">
-        <is>
-          <t>OutputLimitExactBoundaryNotClamped</t>
+      <c r="H57" s="2" t="inlineStr">
+        <is>
+          <t>OutputLimitPassesExactBoundaryThrough</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>PST-17</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>degenerate config</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>zero gains hold zero</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>gains 0, out±5, sp3, fb1</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="inlineStr">
+        <is>
+          <t>0 + int 0</t>
+        </is>
+      </c>
+      <c r="F58" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G58" s="2" t="inlineStr">
+        <is>
+          <t>degenerate</t>
+        </is>
+      </c>
+      <c r="H58" s="2" t="inlineStr">
+        <is>
+          <t>ZeroGainDegenerateConfigHoldsZero</t>
         </is>
       </c>
     </row>
@@ -3448,7 +3714,7 @@
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>PST-02</t>
+          <t>PST-07</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
@@ -3475,12 +3741,12 @@
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>PST-03</t>
+          <t>PST-08</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>c1 independent (only c1 differs vs PST-02)</t>
+          <t>c1 independent (only c1 differs vs PST-07)</t>
         </is>
       </c>
     </row>
@@ -3497,17 +3763,17 @@
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>active ((0.6−0.5)/0.1=1.0 → 5.0)</t>
+          <t>active ((2.5−2.0)/0.5=1.0 → +4.0, PLUS sign L47)</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>PST-04</t>
+          <t>PST-09</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>c2 independent (only c2 differs vs PST-03)</t>
+          <t>c2 independent (only c2 differs vs PST-08)</t>
         </is>
       </c>
     </row>
@@ -3529,7 +3795,7 @@
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>PST-05</t>
+          <t>PST-10</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Option B: add Gyroscope scope (34 tests, 112/112 lines); workbook 95 rows; report + packages resynced
</commit_message>
<xml_diff>
--- a/submission_pkg/24i3102_24i3052_24i3072_C_Workbook.xlsx
+++ b/submission_pkg/24i3102_24i3052_24i3072_C_Workbook.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H62"/>
+  <dimension ref="A1:H96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2349,27 +2349,27 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>PST-01</t>
+          <t>GST-01</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>update + updateIntegral</t>
+          <t>ctor / Reset</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>integral frozen when flag cleared, then evolves</t>
+          <t>default state after construction</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>P2/I5, sp1, fb0, dt0.1, flag F then T</t>
+          <t>fresh object</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>2.0 + int 0; then 2.0 + int 0.5</t>
+          <t>uncalibrated, prio 50, offsets 0</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
@@ -2379,39 +2379,39 @@
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>P-D1 F→T</t>
+          <t>G-D11 internal arm</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>PIDStructural.IntegralFrozenWhenUpdateFlagCleared</t>
+          <t>GyroscopeStructural.DefaultConstructorResetsState</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>PST-02</t>
+          <t>GST-02</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>output clamp + integral</t>
+          <t>device-id ctor</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>high-side saturation clamps output, integral accumulates (no freeze gate in v1.17.0)</t>
+          <t>binds id, no saved cal → Reset</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>I.5/lim10/out±.2, sp2, fb0, dt.5 ×2</t>
+          <t>SIM id</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>0 + int.5; then .2 + int 1.0</t>
+          <t>idx -1, uncalibrated</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
@@ -2421,39 +2421,39 @@
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>saturation edges</t>
+          <t>G-D1 T, G-D9 reset arm</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
-          <t>PIDStructural.SaturationHighClampsOutputIntegralNotFrozen</t>
+          <t>GyroscopeStructural.DeviceIdConstructorBindsWithoutParams</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>PST-03</t>
+          <t>GST-03</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>output clamp + integral</t>
+          <t>set_device_id</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>low-side mirror</t>
+          <t>internal sensor defaults</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>sp−2 mirror</t>
+          <t>SIM id</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>0 + int−.5; then −.2 + int −1.0</t>
+          <t>external F, prio 50</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
@@ -2463,39 +2463,39 @@
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>saturation edges</t>
+          <t>G-D1 T, G-D11 internal</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
-          <t>PIDStructural.SaturationLowClampsOutputIntegralNotFrozen</t>
+          <t>GyroscopeStructural.SetDeviceIdInternalSensor</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>PST-04</t>
+          <t>GST-04</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>integral unwind</t>
+          <t>set_device_id</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>error reversal under saturation unwinds integral</t>
+          <t>external sensor defaults</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>saturated-high, then sp→−2</t>
+          <t>EXT id</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>.2 + int 0.5</t>
+          <t>external T, prio 75</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
@@ -2505,39 +2505,39 @@
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>saturation edges</t>
+          <t>G-D1 T, G-D11 external</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr">
         <is>
-          <t>PIDStructural.SaturationHighThenReversalUnwindsIntegral</t>
+          <t>GyroscopeStructural.SetDeviceIdExternalSensor</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>PST-05</t>
+          <t>GST-05</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>updateIntegral</t>
+          <t>set_device_id</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>NaN feedback discards integral candidate</t>
+          <t>same id keeps state (no Reset)</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>P1/I.1, sp1, fb NaN</t>
+          <t>SIM, offset 0.1, same id again</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>NaN out + int 0; then 0 + int 0</t>
+          <t>offset kept, count 1</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
@@ -2547,39 +2547,39 @@
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>P-D2 F-path</t>
+          <t>G-D1 F-path</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
-          <t>PIDStructural.NonFiniteIntegralCandidateIsDiscarded_NaN</t>
+          <t>GyroscopeStructural.SetDeviceIdSameValueKeepsState</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>PST-06</t>
+          <t>GST-06</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>updateIntegral + output clamp</t>
+          <t>SensorCorrectionsUpdate</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>−Inf feedback clamps output, integral held</t>
+          <t>slot-0 thermal applied</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>P1/I.1, sp1, fb −Inf</t>
+          <t>correction slot 0, SIM</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>+10 + int 0; then 0 + int 0</t>
+          <t>thermal 0.01/0.02/0.03</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
@@ -2589,39 +2589,39 @@
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>P-D2 F-path + clamp</t>
+          <t>G-D2 T, G-D5/G-D6 case 0</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr">
         <is>
-          <t>PIDStructural.NonFiniteIntegralCandidateIsDiscarded_NegInfSaturates</t>
+          <t>GyroscopeStructural.CorrectionIndexZeroApplied</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>PST-07</t>
+          <t>GST-07</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>updateDerivative</t>
+          <t>SensorCorrectionsUpdate</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>guard all-false (dt 0, last NaN)</t>
+          <t>slot-3 thermal applied</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>D4, fb2.0, dt0, fresh</t>
+          <t>correction slot 3, EXT</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>thermal -0.05/0.06/-0.07</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
@@ -2631,39 +2631,39 @@
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>P-D3 FF</t>
+          <t>G-D6 case 3</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr">
         <is>
-          <t>PIDStructural.DerivativeGuardBlocksWhenNoTimeAndNoHistory</t>
+          <t>GyroscopeStructural.CorrectionIndexThreeApplied</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>PST-08</t>
+          <t>GST-08</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>updateDerivative</t>
+          <t>SensorCorrectionsUpdate</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>time ok, no history (dt .5, last NaN)</t>
+          <t>unknown device zeroes thermal</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>D4, fb2.0, dt.5, fresh</t>
+          <t>correction for other id</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>thermal 0</t>
         </is>
       </c>
       <c r="F53" s="2" t="inlineStr">
@@ -2673,39 +2673,39 @@
       </c>
       <c r="G53" s="2" t="inlineStr">
         <is>
-          <t>P-D3 TF</t>
+          <t>G-D5 no-match, L107</t>
         </is>
       </c>
       <c r="H53" s="2" t="inlineStr">
         <is>
-          <t>PIDStructural.DerivativeGuardBlocksWhenTimeOkButNoHistory</t>
+          <t>GyroscopeStructural.CorrectionNotFoundZeroesThermal</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>PST-09</t>
+          <t>GST-09</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>updateDerivative</t>
+          <t>SensorCorrectionsUpdate</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>fully active (PLUS sign, L47)</t>
+          <t>no data + no force → skip</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>D4, seed 2.0/.5, then 2.5/.5</t>
+          <t>nothing published, force F</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>+4.0</t>
+          <t>thermal 0</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
@@ -2715,39 +2715,39 @@
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>P-D3 TT</t>
+          <t>G-D2 F-path</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr">
         <is>
-          <t>PIDStructural.DerivativeGuardActiveWhenTimeAndHistory</t>
+          <t>GyroscopeStructural.NoUpdateWithoutForceOrData</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>PST-10</t>
+          <t>GST-10</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>updateDerivative</t>
+          <t>SensorCorrectionsUpdate</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>history present but dt 0</t>
+          <t>device 0 early return</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>D4, seed 2.0/.5, then 3.0/dt0</t>
+          <t>device 0, force T</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>thermal 0</t>
         </is>
       </c>
       <c r="F55" s="2" t="inlineStr">
@@ -2757,39 +2757,39 @@
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>P-D3 FT</t>
+          <t>G-D3 T</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr">
         <is>
-          <t>PIDStructural.DerivativeGuardBlocksWhenHistoryButNoTime</t>
+          <t>GyroscopeStructural.ZeroDeviceIdSkipsCorrectionCopy</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>PST-11</t>
+          <t>GST-11</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>updateDerivative</t>
+          <t>set_offset</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>exact dt==EPS boundary (not &gt;)</t>
+          <t>first write accepted (count 0)</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>D4, seed 2.0/.5, then 2.5/dt=EPS</t>
+          <t>offset 0.001</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>true, count 1</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
@@ -2799,39 +2799,39 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>P-D3 boundary</t>
+          <t>G-D7 count arm</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
         <is>
-          <t>PIDStructural.DerivativeGuardExactEpsilonIsNotEnoughTime</t>
+          <t>GyroscopeStructural.SetOffsetFirstWriteAccepted</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>PST-12</t>
+          <t>GST-12</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>updateDerivative</t>
+          <t>set_offset</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>just above EPS saturates high via D</t>
+          <t>identical rewrite rejected</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>D4, 2.5/dt=2EPS, lim±100</t>
+          <t>offset 0.1 twice</t>
         </is>
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>+100 (deriv 2097152 exact)</t>
+          <t>second false, count 1</t>
         </is>
       </c>
       <c r="F57" s="2" t="inlineStr">
@@ -2841,39 +2841,39 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>P-D3 T + saturation</t>
+          <t>G-D7 F-path</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
         <is>
-          <t>PIDStructural.DerivativeGuardJustAboveEpsilonSaturatesHigh</t>
+          <t>GyroscopeStructural.SetOffsetSameValueRejected</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>PST-13</t>
+          <t>GST-13</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>updateDerivative</t>
+          <t>set_offset</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>negative dt robustness</t>
+          <t>large change accepted</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>P2/D4, sp1, fb.5, dt−.5</t>
+          <t>0.1 then 0.5</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>1.0 (P-only)</t>
+          <t>true, count 2</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr">
@@ -2883,39 +2883,39 @@
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>P-D3 invalid input</t>
+          <t>G-D7 epsilon arm</t>
         </is>
       </c>
       <c r="H58" s="2" t="inlineStr">
         <is>
-          <t>PIDStructural.NegativeDtDisablesDerivativeTerm</t>
+          <t>GyroscopeStructural.SetOffsetLargeChangeAccepted</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>PST-14</t>
+          <t>GST-14</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>resetDerivative</t>
+          <t>set_offset</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>history cleared to NaN, guard re-entry</t>
+          <t>NaN rejected</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>D2, seed 0/.5, reset, then 1.0/.5</t>
+          <t>NaN offset</t>
         </is>
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>false, count 0</t>
         </is>
       </c>
       <c r="F59" s="2" t="inlineStr">
@@ -2925,39 +2925,39 @@
       </c>
       <c r="G59" s="2" t="inlineStr">
         <is>
-          <t>P-D3 TF re-entry</t>
+          <t>G-D7 finite guard F</t>
         </is>
       </c>
       <c r="H59" s="2" t="inlineStr">
         <is>
-          <t>PIDStructural.ResetDerivativeClearsHistory</t>
+          <t>GyroscopeStructural.SetOffsetRejectsNonFinite</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>PST-15</t>
+          <t>GST-15</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>updateIntegral</t>
+          <t>set_calibration_index</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>windup clamps exactly at limit</t>
+          <t>bounds enforced</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>I1/lim.5/out±10, sp1, fb0, dt.5 ×3</t>
+          <t>2 valid; -1, 4 rejected</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>0, .5, .5; int .5</t>
+          <t>idx stays 2</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr">
@@ -2967,39 +2967,39 @@
       </c>
       <c r="G60" s="2" t="inlineStr">
         <is>
-          <t>P-D1 T + clamp</t>
+          <t>G-D8 T/F</t>
         </is>
       </c>
       <c r="H60" s="2" t="inlineStr">
         <is>
-          <t>PIDStructural.IntegralWindupClampsExactlyAtLimit</t>
+          <t>GyroscopeStructural.SetCalibrationIndexBounds</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>PST-16</t>
+          <t>GST-16</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>output limit</t>
+          <t>ParametersUpdate</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>exact-boundary passthrough + clamp</t>
+          <t>device 0 early return</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>P1/lim±2, sp5, fb 3/2/4</t>
+          <t>fresh object</t>
         </is>
       </c>
       <c r="E61" s="2" t="inlineStr">
         <is>
-          <t>2.0 / 2.0 / 1.0</t>
+          <t>idx -1</t>
         </is>
       </c>
       <c r="F61" s="2" t="inlineStr">
@@ -3009,52 +3009,1480 @@
       </c>
       <c r="G61" s="2" t="inlineStr">
         <is>
-          <t>saturation edges</t>
+          <t>G-D9 L144 T</t>
         </is>
       </c>
       <c r="H61" s="2" t="inlineStr">
         <is>
-          <t>PIDStructural.OutputLimitPassesExactBoundaryThrough</t>
+          <t>GyroscopeStructural.ParametersUpdateNoDeviceReturnsEarly</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
+          <t>GST-17</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>ParametersLoad</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>full valid load, external</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t>slot 0 bound, ROT 2, PRIO 50, OFF set</t>
+        </is>
+      </c>
+      <c r="E62" s="2" t="inlineStr">
+        <is>
+          <t>idx 0, calibrated, ROT 2, prio 50</t>
+        </is>
+      </c>
+      <c r="F62" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G62" s="2" t="inlineStr">
+        <is>
+          <t>G-D9/G-D10 T-paths</t>
+        </is>
+      </c>
+      <c r="H62" s="2" t="inlineStr">
+        <is>
+          <t>GyroscopeStructural.ParametersLoadExternalValid</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>GST-18</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>ParametersLoad</t>
+        </is>
+      </c>
+      <c r="C63" s="2" t="inlineStr">
+        <is>
+          <t>invalid rotation reset</t>
+        </is>
+      </c>
+      <c r="D63" s="2" t="inlineStr">
+        <is>
+          <t>EXT, ROT 99</t>
+        </is>
+      </c>
+      <c r="E63" s="2" t="inlineStr">
+        <is>
+          <t>ROTATION_NONE</t>
+        </is>
+      </c>
+      <c r="F63" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G63" s="2" t="inlineStr">
+        <is>
+          <t>G-D10 L166 T</t>
+        </is>
+      </c>
+      <c r="H63" s="2" t="inlineStr">
+        <is>
+          <t>GyroscopeStructural.InvalidRotationResetToNone</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>GST-19</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>ParametersLoad</t>
+        </is>
+      </c>
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t>invalid priority reset</t>
+        </is>
+      </c>
+      <c r="D64" s="2" t="inlineStr">
+        <is>
+          <t>EXT, PRIO 150</t>
+        </is>
+      </c>
+      <c r="E64" s="2" t="inlineStr">
+        <is>
+          <t>param -1, prio 75</t>
+        </is>
+      </c>
+      <c r="F64" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G64" s="2" t="inlineStr">
+        <is>
+          <t>G-D10 L181/L185 T</t>
+        </is>
+      </c>
+      <c r="H64" s="2" t="inlineStr">
+        <is>
+          <t>GyroscopeStructural.InvalidPriorityResetToDefault</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="inlineStr">
+        <is>
+          <t>GST-20</t>
+        </is>
+      </c>
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>ParametersLoad</t>
+        </is>
+      </c>
+      <c r="C65" s="2" t="inlineStr">
+        <is>
+          <t>internal ignores ROT param</t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="inlineStr">
+        <is>
+          <t>SIM, ROT 2</t>
+        </is>
+      </c>
+      <c r="E65" s="2" t="inlineStr">
+        <is>
+          <t>board rotation</t>
+        </is>
+      </c>
+      <c r="F65" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G65" s="2" t="inlineStr">
+        <is>
+          <t>G-D10 internal arm</t>
+        </is>
+      </c>
+      <c r="H65" s="2" t="inlineStr">
+        <is>
+          <t>GyroscopeStructural.InternalSensorFollowsBoardRotation</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>GST-21</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>ParametersSave</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>forced slot bind</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="inlineStr">
+        <is>
+          <t>EXT unbound, save(1, force)</t>
+        </is>
+      </c>
+      <c r="E66" s="2" t="inlineStr">
+        <is>
+          <t>idx 1, ID param set</t>
+        </is>
+      </c>
+      <c r="F66" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G66" s="2" t="inlineStr">
+        <is>
+          <t>G-D12 L227 T</t>
+        </is>
+      </c>
+      <c r="H66" s="2" t="inlineStr">
+        <is>
+          <t>GyroscopeStructural.ParametersSaveForcedSlot</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="inlineStr">
+        <is>
+          <t>GST-22</t>
+        </is>
+      </c>
+      <c r="B67" s="2" t="inlineStr">
+        <is>
+          <t>ParametersSave</t>
+        </is>
+      </c>
+      <c r="C67" s="2" t="inlineStr">
+        <is>
+          <t>slot moved + warn path</t>
+        </is>
+      </c>
+      <c r="D67" s="2" t="inlineStr">
+        <is>
+          <t>slot 0 rebound elsewhere, save unforced</t>
+        </is>
+      </c>
+      <c r="E67" s="2" t="inlineStr">
+        <is>
+          <t>idx 1</t>
+        </is>
+      </c>
+      <c r="F67" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G67" s="2" t="inlineStr">
+        <is>
+          <t>G-D12 L230 T, L237 warn</t>
+        </is>
+      </c>
+      <c r="H67" s="2" t="inlineStr">
+        <is>
+          <t>GyroscopeStructural.ParametersSaveFindsNewSlotWithWarning</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>GST-23</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>ParametersSave</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>no free slot fails</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="inlineStr">
+        <is>
+          <t>all 4 slots taken, save unforced</t>
+        </is>
+      </c>
+      <c r="E68" s="2" t="inlineStr">
+        <is>
+          <t>false, idx -1</t>
+        </is>
+      </c>
+      <c r="F68" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G68" s="2" t="inlineStr">
+        <is>
+          <t>G-D12 L243 F</t>
+        </is>
+      </c>
+      <c r="H68" s="2" t="inlineStr">
+        <is>
+          <t>GyroscopeStructural.ParametersSaveNoSlotFails</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="inlineStr">
+        <is>
+          <t>GST-24</t>
+        </is>
+      </c>
+      <c r="B69" s="2" t="inlineStr">
+        <is>
+          <t>Correct/Uncorrect</t>
+        </is>
+      </c>
+      <c r="C69" s="2" t="inlineStr">
+        <is>
+          <t>rotation round-trip</t>
+        </is>
+      </c>
+      <c r="D69" s="2" t="inlineStr">
+        <is>
+          <t>SIM, offset set</t>
+        </is>
+      </c>
+      <c r="E69" s="2" t="inlineStr">
+        <is>
+          <t>back == raw</t>
+        </is>
+      </c>
+      <c r="F69" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G69" s="2" t="inlineStr">
+        <is>
+          <t>inline math</t>
+        </is>
+      </c>
+      <c r="H69" s="2" t="inlineStr">
+        <is>
+          <t>GyroscopeStructural.CorrectUncorrectRoundTrip</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>GST-25</t>
+        </is>
+      </c>
+      <c r="B70" s="2" t="inlineStr">
+        <is>
+          <t>BiasCorrectedSensorOffset</t>
+        </is>
+      </c>
+      <c r="C70" s="2" t="inlineStr">
+        <is>
+          <t>bias math</t>
+        </is>
+      </c>
+      <c r="D70" s="2" t="inlineStr">
+        <is>
+          <t>SIM, offset + bias</t>
+        </is>
+      </c>
+      <c r="E70" s="2" t="inlineStr">
+        <is>
+          <t>offset + Rᵀ·bias</t>
+        </is>
+      </c>
+      <c r="F70" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G70" s="2" t="inlineStr">
+        <is>
+          <t>inline math</t>
+        </is>
+      </c>
+      <c r="H70" s="2" t="inlineStr">
+        <is>
+          <t>GyroscopeStructural.BiasCorrectedSensorOffsetMath</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t>GST-26</t>
+        </is>
+      </c>
+      <c r="B71" s="2" t="inlineStr">
+        <is>
+          <t>PrintStatus</t>
+        </is>
+      </c>
+      <c r="C71" s="2" t="inlineStr">
+        <is>
+          <t>external/internal + thermal log arms</t>
+        </is>
+      </c>
+      <c r="D71" s="2" t="inlineStr">
+        <is>
+          <t>EXT w/ thermal; SIM</t>
+        </is>
+      </c>
+      <c r="E71" s="2" t="inlineStr">
+        <is>
+          <t>no crash</t>
+        </is>
+      </c>
+      <c r="F71" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G71" s="2" t="inlineStr">
+        <is>
+          <t>G-D13 both</t>
+        </is>
+      </c>
+      <c r="H71" s="2" t="inlineStr">
+        <is>
+          <t>GyroscopeStructural.PrintStatusBothPaths</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>GST-27</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="inlineStr">
+        <is>
+          <t>SensorCorrectionsUpdate</t>
+        </is>
+      </c>
+      <c r="C72" s="2" t="inlineStr">
+        <is>
+          <t>slot-2 thermal applied</t>
+        </is>
+      </c>
+      <c r="D72" s="2" t="inlineStr">
+        <is>
+          <t>correction slot 2, SIM2</t>
+        </is>
+      </c>
+      <c r="E72" s="2" t="inlineStr">
+        <is>
+          <t>thermal 0.04/-0.05/0.06</t>
+        </is>
+      </c>
+      <c r="F72" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G72" s="2" t="inlineStr">
+        <is>
+          <t>G-D6 case 2 (L95-97)</t>
+        </is>
+      </c>
+      <c r="H72" s="2" t="inlineStr">
+        <is>
+          <t>GyroscopeStructural.CorrectionSlotTwoApplied</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="inlineStr">
+        <is>
+          <t>GST-28</t>
+        </is>
+      </c>
+      <c r="B73" s="2" t="inlineStr">
+        <is>
+          <t>ParametersLoad</t>
+        </is>
+      </c>
+      <c r="C73" s="2" t="inlineStr">
+        <is>
+          <t>direct call, index -1 → false</t>
+        </is>
+      </c>
+      <c r="D73" s="2" t="inlineStr">
+        <is>
+          <t>fresh object Load()</t>
+        </is>
+      </c>
+      <c r="E73" s="2" t="inlineStr">
+        <is>
+          <t>false, idx -1</t>
+        </is>
+      </c>
+      <c r="F73" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G73" s="2" t="inlineStr">
+        <is>
+          <t>G-D10 L161 F, L201</t>
+        </is>
+      </c>
+      <c r="H73" s="2" t="inlineStr">
+        <is>
+          <t>GyroscopeStructural.ParametersLoadRejectedIndexDirect</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>GST-29</t>
+        </is>
+      </c>
+      <c r="B74" s="2" t="inlineStr">
+        <is>
+          <t>ParametersSave</t>
+        </is>
+      </c>
+      <c r="C74" s="2" t="inlineStr">
+        <is>
+          <t>forced negative desired → slot kept</t>
+        </is>
+      </c>
+      <c r="D74" s="2" t="inlineStr">
+        <is>
+          <t>bound idx 0, save(-1, force)</t>
+        </is>
+      </c>
+      <c r="E74" s="2" t="inlineStr">
+        <is>
+          <t>idx 0, success</t>
+        </is>
+      </c>
+      <c r="F74" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G74" s="2" t="inlineStr">
+        <is>
+          <t>G-D12 L227 F, L230-231 F</t>
+        </is>
+      </c>
+      <c r="H74" s="2" t="inlineStr">
+        <is>
+          <t>GyroscopeStructural.SaveForcedNegativeDesiredFindsSlot</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="inlineStr">
+        <is>
+          <t>GST-30</t>
+        </is>
+      </c>
+      <c r="B75" s="2" t="inlineStr">
+        <is>
+          <t>ParametersSave</t>
+        </is>
+      </c>
+      <c r="C75" s="2" t="inlineStr">
+        <is>
+          <t>internal ROT=-1 marker saved</t>
+        </is>
+      </c>
+      <c r="D75" s="2" t="inlineStr">
+        <is>
+          <t>SIM bound, save unforced then forced</t>
+        </is>
+      </c>
+      <c r="E75" s="2" t="inlineStr">
+        <is>
+          <t>ROT param -1</t>
+        </is>
+      </c>
+      <c r="F75" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G75" s="2" t="inlineStr">
+        <is>
+          <t>G-D12 L237 no-warn, L253-254</t>
+        </is>
+      </c>
+      <c r="H75" s="2" t="inlineStr">
+        <is>
+          <t>GyroscopeStructural.SaveInternalWritesRotationMinusOne</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="inlineStr">
+        <is>
+          <t>GST-31</t>
+        </is>
+      </c>
+      <c r="B76" s="2" t="inlineStr">
+        <is>
+          <t>SensorCorrectionsUpdate</t>
+        </is>
+      </c>
+      <c r="C76" s="2" t="inlineStr">
+        <is>
+          <t>unadvertised topic skips copy</t>
+        </is>
+      </c>
+      <c r="D76" s="2" t="inlineStr">
+        <is>
+          <t>publish, unadvertise, fresh gyro</t>
+        </is>
+      </c>
+      <c r="E76" s="2" t="inlineStr">
+        <is>
+          <t>thermal 0</t>
+        </is>
+      </c>
+      <c r="F76" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G76" s="2" t="inlineStr">
+        <is>
+          <t>G-D2 robustness (L84-F)</t>
+        </is>
+      </c>
+      <c r="H76" s="2" t="inlineStr">
+        <is>
+          <t>GyroscopeStructural.UnadvertisedCorrectionSkipsCopy</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="inlineStr">
+        <is>
+          <t>GST-32</t>
+        </is>
+      </c>
+      <c r="B77" s="2" t="inlineStr">
+        <is>
+          <t>ParametersSave</t>
+        </is>
+      </c>
+      <c r="C77" s="2" t="inlineStr">
+        <is>
+          <t>out-of-range desired → free slot</t>
+        </is>
+      </c>
+      <c r="D77" s="2" t="inlineStr">
+        <is>
+          <t>unbound, save(4, force)</t>
+        </is>
+      </c>
+      <c r="E77" s="2" t="inlineStr">
+        <is>
+          <t>idx 0, success</t>
+        </is>
+      </c>
+      <c r="F77" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G77" s="2" t="inlineStr">
+        <is>
+          <t>G-D12 L227 3rd-op F</t>
+        </is>
+      </c>
+      <c r="H77" s="2" t="inlineStr">
+        <is>
+          <t>GyroscopeStructural.SaveOutOfRangeDesiredFallsBackToFreeSlot</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t>GST-33</t>
+        </is>
+      </c>
+      <c r="B78" s="2" t="inlineStr">
+        <is>
+          <t>ParametersSave</t>
+        </is>
+      </c>
+      <c r="C78" s="2" t="inlineStr">
+        <is>
+          <t>unbound + force resolves slot</t>
+        </is>
+      </c>
+      <c r="D78" s="2" t="inlineStr">
+        <is>
+          <t>device 0, save(-1, force)</t>
+        </is>
+      </c>
+      <c r="E78" s="2" t="inlineStr">
+        <is>
+          <t>idx 0, success</t>
+        </is>
+      </c>
+      <c r="F78" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G78" s="2" t="inlineStr">
+        <is>
+          <t>G-D12 L230 2nd-op T</t>
+        </is>
+      </c>
+      <c r="H78" s="2" t="inlineStr">
+        <is>
+          <t>GyroscopeStructural.SaveUnboundNegativeDesiredFindsSlot</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="inlineStr">
+        <is>
+          <t>GST-34</t>
+        </is>
+      </c>
+      <c r="B79" s="2" t="inlineStr">
+        <is>
+          <t>ParametersSave</t>
+        </is>
+      </c>
+      <c r="C79" s="2" t="inlineStr">
+        <is>
+          <t>out-of-range desired keeps bound slot</t>
+        </is>
+      </c>
+      <c r="D79" s="2" t="inlineStr">
+        <is>
+          <t>bound idx 0, save(4, force)</t>
+        </is>
+      </c>
+      <c r="E79" s="2" t="inlineStr">
+        <is>
+          <t>idx 0, success</t>
+        </is>
+      </c>
+      <c r="F79" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G79" s="2" t="inlineStr">
+        <is>
+          <t>G-D12 L231 full eval</t>
+        </is>
+      </c>
+      <c r="H79" s="2" t="inlineStr">
+        <is>
+          <t>GyroscopeStructural.SaveOutOfRangeDesiredKeepsBoundSlot</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="inlineStr">
+        <is>
+          <t>PST-01</t>
+        </is>
+      </c>
+      <c r="B80" s="2" t="inlineStr">
+        <is>
+          <t>update + updateIntegral</t>
+        </is>
+      </c>
+      <c r="C80" s="2" t="inlineStr">
+        <is>
+          <t>integral frozen when flag cleared, then evolves</t>
+        </is>
+      </c>
+      <c r="D80" s="2" t="inlineStr">
+        <is>
+          <t>P2/I5, sp1, fb0, dt0.1, flag F then T</t>
+        </is>
+      </c>
+      <c r="E80" s="2" t="inlineStr">
+        <is>
+          <t>2.0 + int 0; then 2.0 + int 0.5</t>
+        </is>
+      </c>
+      <c r="F80" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G80" s="2" t="inlineStr">
+        <is>
+          <t>P-D1 F→T</t>
+        </is>
+      </c>
+      <c r="H80" s="2" t="inlineStr">
+        <is>
+          <t>PIDStructural.IntegralFrozenWhenUpdateFlagCleared</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="inlineStr">
+        <is>
+          <t>PST-02</t>
+        </is>
+      </c>
+      <c r="B81" s="2" t="inlineStr">
+        <is>
+          <t>output clamp + integral</t>
+        </is>
+      </c>
+      <c r="C81" s="2" t="inlineStr">
+        <is>
+          <t>high-side saturation clamps output, integral accumulates (no freeze gate in v1.17.0)</t>
+        </is>
+      </c>
+      <c r="D81" s="2" t="inlineStr">
+        <is>
+          <t>I.5/lim10/out±.2, sp2, fb0, dt.5 ×2</t>
+        </is>
+      </c>
+      <c r="E81" s="2" t="inlineStr">
+        <is>
+          <t>0 + int.5; then .2 + int 1.0</t>
+        </is>
+      </c>
+      <c r="F81" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G81" s="2" t="inlineStr">
+        <is>
+          <t>saturation edges</t>
+        </is>
+      </c>
+      <c r="H81" s="2" t="inlineStr">
+        <is>
+          <t>PIDStructural.SaturationHighClampsOutputIntegralNotFrozen</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>PST-03</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>output clamp + integral</t>
+        </is>
+      </c>
+      <c r="C82" s="2" t="inlineStr">
+        <is>
+          <t>low-side mirror</t>
+        </is>
+      </c>
+      <c r="D82" s="2" t="inlineStr">
+        <is>
+          <t>sp−2 mirror</t>
+        </is>
+      </c>
+      <c r="E82" s="2" t="inlineStr">
+        <is>
+          <t>0 + int−.5; then −.2 + int −1.0</t>
+        </is>
+      </c>
+      <c r="F82" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G82" s="2" t="inlineStr">
+        <is>
+          <t>saturation edges</t>
+        </is>
+      </c>
+      <c r="H82" s="2" t="inlineStr">
+        <is>
+          <t>PIDStructural.SaturationLowClampsOutputIntegralNotFrozen</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="inlineStr">
+        <is>
+          <t>PST-04</t>
+        </is>
+      </c>
+      <c r="B83" s="2" t="inlineStr">
+        <is>
+          <t>integral unwind</t>
+        </is>
+      </c>
+      <c r="C83" s="2" t="inlineStr">
+        <is>
+          <t>error reversal under saturation unwinds integral</t>
+        </is>
+      </c>
+      <c r="D83" s="2" t="inlineStr">
+        <is>
+          <t>saturated-high, then sp→−2</t>
+        </is>
+      </c>
+      <c r="E83" s="2" t="inlineStr">
+        <is>
+          <t>.2 + int 0.5</t>
+        </is>
+      </c>
+      <c r="F83" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G83" s="2" t="inlineStr">
+        <is>
+          <t>saturation edges</t>
+        </is>
+      </c>
+      <c r="H83" s="2" t="inlineStr">
+        <is>
+          <t>PIDStructural.SaturationHighThenReversalUnwindsIntegral</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="inlineStr">
+        <is>
+          <t>PST-05</t>
+        </is>
+      </c>
+      <c r="B84" s="2" t="inlineStr">
+        <is>
+          <t>updateIntegral</t>
+        </is>
+      </c>
+      <c r="C84" s="2" t="inlineStr">
+        <is>
+          <t>NaN feedback discards integral candidate</t>
+        </is>
+      </c>
+      <c r="D84" s="2" t="inlineStr">
+        <is>
+          <t>P1/I.1, sp1, fb NaN</t>
+        </is>
+      </c>
+      <c r="E84" s="2" t="inlineStr">
+        <is>
+          <t>NaN out + int 0; then 0 + int 0</t>
+        </is>
+      </c>
+      <c r="F84" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G84" s="2" t="inlineStr">
+        <is>
+          <t>P-D2 F-path</t>
+        </is>
+      </c>
+      <c r="H84" s="2" t="inlineStr">
+        <is>
+          <t>PIDStructural.NonFiniteIntegralCandidateIsDiscarded_NaN</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="inlineStr">
+        <is>
+          <t>PST-06</t>
+        </is>
+      </c>
+      <c r="B85" s="2" t="inlineStr">
+        <is>
+          <t>updateIntegral + output clamp</t>
+        </is>
+      </c>
+      <c r="C85" s="2" t="inlineStr">
+        <is>
+          <t>−Inf feedback clamps output, integral held</t>
+        </is>
+      </c>
+      <c r="D85" s="2" t="inlineStr">
+        <is>
+          <t>P1/I.1, sp1, fb −Inf</t>
+        </is>
+      </c>
+      <c r="E85" s="2" t="inlineStr">
+        <is>
+          <t>+10 + int 0; then 0 + int 0</t>
+        </is>
+      </c>
+      <c r="F85" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G85" s="2" t="inlineStr">
+        <is>
+          <t>P-D2 F-path + clamp</t>
+        </is>
+      </c>
+      <c r="H85" s="2" t="inlineStr">
+        <is>
+          <t>PIDStructural.NonFiniteIntegralCandidateIsDiscarded_NegInfSaturates</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="inlineStr">
+        <is>
+          <t>PST-07</t>
+        </is>
+      </c>
+      <c r="B86" s="2" t="inlineStr">
+        <is>
+          <t>updateDerivative</t>
+        </is>
+      </c>
+      <c r="C86" s="2" t="inlineStr">
+        <is>
+          <t>guard all-false (dt 0, last NaN)</t>
+        </is>
+      </c>
+      <c r="D86" s="2" t="inlineStr">
+        <is>
+          <t>D4, fb2.0, dt0, fresh</t>
+        </is>
+      </c>
+      <c r="E86" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F86" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G86" s="2" t="inlineStr">
+        <is>
+          <t>P-D3 FF</t>
+        </is>
+      </c>
+      <c r="H86" s="2" t="inlineStr">
+        <is>
+          <t>PIDStructural.DerivativeGuardBlocksWhenNoTimeAndNoHistory</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="inlineStr">
+        <is>
+          <t>PST-08</t>
+        </is>
+      </c>
+      <c r="B87" s="2" t="inlineStr">
+        <is>
+          <t>updateDerivative</t>
+        </is>
+      </c>
+      <c r="C87" s="2" t="inlineStr">
+        <is>
+          <t>time ok, no history (dt .5, last NaN)</t>
+        </is>
+      </c>
+      <c r="D87" s="2" t="inlineStr">
+        <is>
+          <t>D4, fb2.0, dt.5, fresh</t>
+        </is>
+      </c>
+      <c r="E87" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F87" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G87" s="2" t="inlineStr">
+        <is>
+          <t>P-D3 TF</t>
+        </is>
+      </c>
+      <c r="H87" s="2" t="inlineStr">
+        <is>
+          <t>PIDStructural.DerivativeGuardBlocksWhenTimeOkButNoHistory</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="inlineStr">
+        <is>
+          <t>PST-09</t>
+        </is>
+      </c>
+      <c r="B88" s="2" t="inlineStr">
+        <is>
+          <t>updateDerivative</t>
+        </is>
+      </c>
+      <c r="C88" s="2" t="inlineStr">
+        <is>
+          <t>fully active (PLUS sign, L47)</t>
+        </is>
+      </c>
+      <c r="D88" s="2" t="inlineStr">
+        <is>
+          <t>D4, seed 2.0/.5, then 2.5/.5</t>
+        </is>
+      </c>
+      <c r="E88" s="2" t="inlineStr">
+        <is>
+          <t>+4.0</t>
+        </is>
+      </c>
+      <c r="F88" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G88" s="2" t="inlineStr">
+        <is>
+          <t>P-D3 TT</t>
+        </is>
+      </c>
+      <c r="H88" s="2" t="inlineStr">
+        <is>
+          <t>PIDStructural.DerivativeGuardActiveWhenTimeAndHistory</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="inlineStr">
+        <is>
+          <t>PST-10</t>
+        </is>
+      </c>
+      <c r="B89" s="2" t="inlineStr">
+        <is>
+          <t>updateDerivative</t>
+        </is>
+      </c>
+      <c r="C89" s="2" t="inlineStr">
+        <is>
+          <t>history present but dt 0</t>
+        </is>
+      </c>
+      <c r="D89" s="2" t="inlineStr">
+        <is>
+          <t>D4, seed 2.0/.5, then 3.0/dt0</t>
+        </is>
+      </c>
+      <c r="E89" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F89" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G89" s="2" t="inlineStr">
+        <is>
+          <t>P-D3 FT</t>
+        </is>
+      </c>
+      <c r="H89" s="2" t="inlineStr">
+        <is>
+          <t>PIDStructural.DerivativeGuardBlocksWhenHistoryButNoTime</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="inlineStr">
+        <is>
+          <t>PST-11</t>
+        </is>
+      </c>
+      <c r="B90" s="2" t="inlineStr">
+        <is>
+          <t>updateDerivative</t>
+        </is>
+      </c>
+      <c r="C90" s="2" t="inlineStr">
+        <is>
+          <t>exact dt==EPS boundary (not &gt;)</t>
+        </is>
+      </c>
+      <c r="D90" s="2" t="inlineStr">
+        <is>
+          <t>D4, seed 2.0/.5, then 2.5/dt=EPS</t>
+        </is>
+      </c>
+      <c r="E90" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F90" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G90" s="2" t="inlineStr">
+        <is>
+          <t>P-D3 boundary</t>
+        </is>
+      </c>
+      <c r="H90" s="2" t="inlineStr">
+        <is>
+          <t>PIDStructural.DerivativeGuardExactEpsilonIsNotEnoughTime</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="inlineStr">
+        <is>
+          <t>PST-12</t>
+        </is>
+      </c>
+      <c r="B91" s="2" t="inlineStr">
+        <is>
+          <t>updateDerivative</t>
+        </is>
+      </c>
+      <c r="C91" s="2" t="inlineStr">
+        <is>
+          <t>just above EPS saturates high via D</t>
+        </is>
+      </c>
+      <c r="D91" s="2" t="inlineStr">
+        <is>
+          <t>D4, 2.5/dt=2EPS, lim±100</t>
+        </is>
+      </c>
+      <c r="E91" s="2" t="inlineStr">
+        <is>
+          <t>+100 (deriv 2097152 exact)</t>
+        </is>
+      </c>
+      <c r="F91" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G91" s="2" t="inlineStr">
+        <is>
+          <t>P-D3 T + saturation</t>
+        </is>
+      </c>
+      <c r="H91" s="2" t="inlineStr">
+        <is>
+          <t>PIDStructural.DerivativeGuardJustAboveEpsilonSaturatesHigh</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="inlineStr">
+        <is>
+          <t>PST-13</t>
+        </is>
+      </c>
+      <c r="B92" s="2" t="inlineStr">
+        <is>
+          <t>updateDerivative</t>
+        </is>
+      </c>
+      <c r="C92" s="2" t="inlineStr">
+        <is>
+          <t>negative dt robustness</t>
+        </is>
+      </c>
+      <c r="D92" s="2" t="inlineStr">
+        <is>
+          <t>P2/D4, sp1, fb.5, dt−.5</t>
+        </is>
+      </c>
+      <c r="E92" s="2" t="inlineStr">
+        <is>
+          <t>1.0 (P-only)</t>
+        </is>
+      </c>
+      <c r="F92" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G92" s="2" t="inlineStr">
+        <is>
+          <t>P-D3 invalid input</t>
+        </is>
+      </c>
+      <c r="H92" s="2" t="inlineStr">
+        <is>
+          <t>PIDStructural.NegativeDtDisablesDerivativeTerm</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="inlineStr">
+        <is>
+          <t>PST-14</t>
+        </is>
+      </c>
+      <c r="B93" s="2" t="inlineStr">
+        <is>
+          <t>resetDerivative</t>
+        </is>
+      </c>
+      <c r="C93" s="2" t="inlineStr">
+        <is>
+          <t>history cleared to NaN, guard re-entry</t>
+        </is>
+      </c>
+      <c r="D93" s="2" t="inlineStr">
+        <is>
+          <t>D2, seed 0/.5, reset, then 1.0/.5</t>
+        </is>
+      </c>
+      <c r="E93" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F93" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G93" s="2" t="inlineStr">
+        <is>
+          <t>P-D3 TF re-entry</t>
+        </is>
+      </c>
+      <c r="H93" s="2" t="inlineStr">
+        <is>
+          <t>PIDStructural.ResetDerivativeClearsHistory</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="inlineStr">
+        <is>
+          <t>PST-15</t>
+        </is>
+      </c>
+      <c r="B94" s="2" t="inlineStr">
+        <is>
+          <t>updateIntegral</t>
+        </is>
+      </c>
+      <c r="C94" s="2" t="inlineStr">
+        <is>
+          <t>windup clamps exactly at limit</t>
+        </is>
+      </c>
+      <c r="D94" s="2" t="inlineStr">
+        <is>
+          <t>I1/lim.5/out±10, sp1, fb0, dt.5 ×3</t>
+        </is>
+      </c>
+      <c r="E94" s="2" t="inlineStr">
+        <is>
+          <t>0, .5, .5; int .5</t>
+        </is>
+      </c>
+      <c r="F94" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G94" s="2" t="inlineStr">
+        <is>
+          <t>P-D1 T + clamp</t>
+        </is>
+      </c>
+      <c r="H94" s="2" t="inlineStr">
+        <is>
+          <t>PIDStructural.IntegralWindupClampsExactlyAtLimit</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="inlineStr">
+        <is>
+          <t>PST-16</t>
+        </is>
+      </c>
+      <c r="B95" s="2" t="inlineStr">
+        <is>
+          <t>output limit</t>
+        </is>
+      </c>
+      <c r="C95" s="2" t="inlineStr">
+        <is>
+          <t>exact-boundary passthrough + clamp</t>
+        </is>
+      </c>
+      <c r="D95" s="2" t="inlineStr">
+        <is>
+          <t>P1/lim±2, sp5, fb 3/2/4</t>
+        </is>
+      </c>
+      <c r="E95" s="2" t="inlineStr">
+        <is>
+          <t>2.0 / 2.0 / 1.0</t>
+        </is>
+      </c>
+      <c r="F95" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G95" s="2" t="inlineStr">
+        <is>
+          <t>saturation edges</t>
+        </is>
+      </c>
+      <c r="H95" s="2" t="inlineStr">
+        <is>
+          <t>PIDStructural.OutputLimitPassesExactBoundaryThrough</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="inlineStr">
+        <is>
           <t>PST-17</t>
         </is>
       </c>
-      <c r="B62" s="2" t="inlineStr">
+      <c r="B96" s="2" t="inlineStr">
         <is>
           <t>degenerate config</t>
         </is>
       </c>
-      <c r="C62" s="2" t="inlineStr">
+      <c r="C96" s="2" t="inlineStr">
         <is>
           <t>zero gains hold zero</t>
         </is>
       </c>
-      <c r="D62" s="2" t="inlineStr">
+      <c r="D96" s="2" t="inlineStr">
         <is>
           <t>gains 0, out±5, sp3, fb1</t>
         </is>
       </c>
-      <c r="E62" s="2" t="inlineStr">
+      <c r="E96" s="2" t="inlineStr">
         <is>
           <t>0 + int 0</t>
         </is>
       </c>
-      <c r="F62" s="2" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="G62" s="2" t="inlineStr">
+      <c r="F96" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G96" s="2" t="inlineStr">
         <is>
           <t>degenerate</t>
         </is>
       </c>
-      <c r="H62" s="2" t="inlineStr">
+      <c r="H96" s="2" t="inlineStr">
         <is>
           <t>PIDStructural.ZeroGainDegenerateConfigHoldsZero</t>
         </is>

</xml_diff>